<commit_message>
Add Pine Point + update Scarborough Beach SE based on real-world observation
</commit_message>
<xml_diff>
--- a/East_Coast_Surf_Spots.xlsx
+++ b/East_Coast_Surf_Spots.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="131">
   <si>
     <t xml:space="preserve">🏄  East Coast Surf Spots — Maine Database</t>
   </si>
@@ -174,7 +174,7 @@
     <t xml:space="preserve">Med</t>
   </si>
   <si>
-    <t xml:space="preserve">State park beach. Can produce punchy surf after NE storms. Parking fee in-season. Closes in winter.</t>
+    <t xml:space="preserve">State park beach. Faces SE — picks up SSE swell well (better angle than Pine Point on SSE days). Prouts Neck focuses energy into beach on SE/SSE. Also works NE/E. Parking fee in-season. Closes in winter. Source: real-world observation, May 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Fortunes Rocks Beach</t>
@@ -289,6 +289,12 @@
   </si>
   <si>
     <t xml:space="preserve">Small crescent beach in York village. Surrounded by buildings which can block wind. Works at all tides. Can get crowded – popular tourist beach. Limited parking.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pine Point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">River mouth setup at the Scarborough River. Shifting sandbars create punchy, hollow peaks — similar feel to Ogunquit Rivermouth. Sits inside Saco Bay which creates a shadow on SSE swell (loses energy vs Scarborough Beach on SSE days). Fires on NE/E groundswell when the river mouth banks line up. Best at low tide when sandbars are exposed. Source: real-world observation, May 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">🌊  Swell Finder — Best Spots for Today's Conditions</t>
@@ -552,6 +558,12 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF888888"/>
@@ -571,12 +583,6 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF1B3A5C"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -705,11 +711,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -798,11 +808,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -810,19 +828,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="21" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -839,7 +857,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="18">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -907,6 +925,13 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FF999999"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -941,6 +966,35 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFE8873A"/>
           <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF375623"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <color rgb="FF999999"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1049,34 +1103,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1222,994 +1276,1056 @@
     <tabColor rgb="FF1B3A5C"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="P3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="Q3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="R3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="S3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="T3" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L4" s="6" t="s">
+      <c r="F4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="O4" s="6" t="s">
+      <c r="O4" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="P4" s="6" t="s">
+      <c r="P4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="Q4" s="6" t="s">
+      <c r="Q4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="R4" s="6" t="s">
+      <c r="R4" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="S4" s="10" t="s">
+      <c r="S4" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="T4" s="11" t="s">
+      <c r="T4" s="12" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L5" s="12" t="s">
+      <c r="F5" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L5" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="M5" s="12" t="s">
+      <c r="M5" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="N5" s="12" t="s">
+      <c r="N5" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="O5" s="12" t="s">
+      <c r="O5" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="P5" s="12" t="s">
+      <c r="P5" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="Q5" s="12" t="s">
+      <c r="Q5" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="R5" s="12" t="s">
+      <c r="R5" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="S5" s="13" t="s">
+      <c r="S5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="T5" s="11" t="s">
+      <c r="T5" s="12" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L6" s="6" t="s">
+      <c r="F6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="M6" s="6" t="s">
+      <c r="M6" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="N6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="O6" s="6" t="s">
+      <c r="O6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="P6" s="6" t="s">
+      <c r="P6" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="Q6" s="6" t="s">
+      <c r="Q6" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="R6" s="6" t="s">
+      <c r="R6" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="S6" s="14" t="s">
+      <c r="S6" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="T6" s="11" t="s">
+      <c r="T6" s="12" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L7" s="12" t="s">
+      <c r="F7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L7" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="M7" s="12" t="s">
+      <c r="M7" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="N7" s="12" t="s">
+      <c r="N7" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="O7" s="12" t="s">
+      <c r="O7" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="P7" s="12" t="s">
+      <c r="P7" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="Q7" s="12" t="s">
+      <c r="Q7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="R7" s="12" t="s">
+      <c r="R7" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="S7" s="13" t="s">
+      <c r="S7" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="T7" s="11" t="s">
+      <c r="T7" s="12" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L8" s="6" t="s">
+      <c r="F8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="M8" s="6" t="s">
+      <c r="M8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="N8" s="6" t="s">
+      <c r="N8" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="O8" s="6" t="s">
+      <c r="O8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="P8" s="6" t="s">
+      <c r="P8" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="Q8" s="6" t="s">
+      <c r="Q8" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="R8" s="6" t="s">
+      <c r="R8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="S8" s="14" t="s">
+      <c r="S8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="T8" s="11" t="s">
+      <c r="T8" s="12" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L9" s="12" t="s">
+      <c r="F9" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L9" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="M9" s="12" t="s">
+      <c r="M9" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="N9" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="O9" s="12" t="s">
+      <c r="O9" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="P9" s="12" t="s">
+      <c r="P9" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="Q9" s="12" t="s">
+      <c r="Q9" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="R9" s="12" t="s">
+      <c r="R9" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="S9" s="13" t="s">
+      <c r="S9" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="T9" s="11" t="s">
+      <c r="T9" s="12" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L10" s="6" t="s">
+      <c r="F10" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="M10" s="6" t="s">
+      <c r="M10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="N10" s="6" t="s">
+      <c r="N10" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="O10" s="6" t="s">
+      <c r="O10" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="P10" s="6" t="s">
+      <c r="P10" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="Q10" s="6" t="s">
+      <c r="Q10" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="R10" s="6" t="s">
+      <c r="R10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="S10" s="10" t="s">
+      <c r="S10" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="T10" s="11" t="s">
+      <c r="T10" s="12" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="12" t="s">
+      <c r="A11" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L11" s="12" t="s">
+      <c r="F11" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="M11" s="12" t="s">
+      <c r="M11" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="N11" s="12" t="s">
+      <c r="N11" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="O11" s="12" t="s">
+      <c r="O11" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="P11" s="12" t="s">
+      <c r="P11" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="Q11" s="12" t="s">
+      <c r="Q11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="R11" s="12" t="s">
+      <c r="R11" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="S11" s="16" t="s">
+      <c r="S11" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="T11" s="11" t="s">
+      <c r="T11" s="12" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K12" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L12" s="6" t="s">
+      <c r="F12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="M12" s="6" t="s">
+      <c r="M12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="N12" s="6" t="s">
+      <c r="N12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="O12" s="6" t="s">
+      <c r="O12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="P12" s="6" t="s">
+      <c r="P12" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="Q12" s="6" t="s">
+      <c r="Q12" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="R12" s="6" t="s">
+      <c r="R12" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="S12" s="14" t="s">
+      <c r="S12" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="T12" s="11" t="s">
+      <c r="T12" s="12" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L13" s="12" t="s">
+      <c r="F13" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L13" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="M13" s="12" t="s">
+      <c r="M13" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="N13" s="12" t="s">
+      <c r="N13" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="O13" s="12" t="s">
+      <c r="O13" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="P13" s="12" t="s">
+      <c r="P13" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="Q13" s="12" t="s">
+      <c r="Q13" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="R13" s="12" t="s">
+      <c r="R13" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="S13" s="13" t="s">
+      <c r="S13" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="T13" s="11" t="s">
+      <c r="T13" s="12" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J14" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L14" s="6" t="s">
+      <c r="F14" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="M14" s="6" t="s">
+      <c r="M14" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="N14" s="6" t="s">
+      <c r="N14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="O14" s="6" t="s">
+      <c r="O14" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="P14" s="6" t="s">
+      <c r="P14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="Q14" s="6" t="s">
+      <c r="Q14" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="R14" s="6" t="s">
+      <c r="R14" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="S14" s="14" t="s">
+      <c r="S14" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="T14" s="11" t="s">
+      <c r="T14" s="12" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F15" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K15" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L15" s="12" t="s">
+      <c r="F15" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L15" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="M15" s="12" t="s">
+      <c r="M15" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="N15" s="12" t="s">
+      <c r="N15" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="O15" s="12" t="s">
+      <c r="O15" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="P15" s="12" t="s">
+      <c r="P15" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="Q15" s="12" t="s">
+      <c r="Q15" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="R15" s="12" t="s">
+      <c r="R15" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="S15" s="16" t="s">
+      <c r="S15" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="T15" s="11" t="s">
+      <c r="T15" s="12" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F16" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J16" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K16" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L16" s="6" t="s">
+      <c r="F16" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L16" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="M16" s="6" t="s">
+      <c r="M16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="N16" s="6" t="s">
+      <c r="N16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="O16" s="6" t="s">
+      <c r="O16" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="P16" s="6" t="s">
+      <c r="P16" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="Q16" s="6" t="s">
+      <c r="Q16" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="R16" s="6" t="s">
+      <c r="R16" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="S16" s="10" t="s">
+      <c r="S16" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="T16" s="11" t="s">
+      <c r="T16" s="12" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="F17" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K17" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L17" s="12" t="s">
+      <c r="F17" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L17" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="M17" s="12" t="s">
+      <c r="M17" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="N17" s="12" t="s">
+      <c r="N17" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="O17" s="12" t="s">
+      <c r="O17" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="P17" s="12" t="s">
+      <c r="P17" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="Q17" s="12" t="s">
+      <c r="Q17" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="R17" s="12" t="s">
+      <c r="R17" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="S17" s="13" t="s">
+      <c r="S17" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="T17" s="11" t="s">
+      <c r="T17" s="12" t="s">
         <v>87</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K18" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="R18" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="S18" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="T18" s="12" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -2239,636 +2355,673 @@
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="A1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
+      <c r="A2" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="19" t="s">
+      <c r="A4" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="C4" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="D4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" s="20" t="s">
+      <c r="A7" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="20" t="s">
+      <c r="I7" s="21" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="str">
+      <c r="A8" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F4="Y"),AND($C$4="NE",'Spots Database'!G4="Y"),AND($C$4="E",'Spots Database'!H4="Y"),AND($C$4="SE",'Spots Database'!I4="Y"),AND($C$4="S",'Spots Database'!J4="Y"),AND($C$4="SW",'Spots Database'!K4="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B8" s="22" t="str">
+      <c r="B8" s="23" t="str">
         <f aca="false">'Spots Database'!S4</f>
         <v>★★★★☆</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="7" t="str">
         <f aca="false">'Spots Database'!B4</f>
         <v>Higgins Beach</v>
       </c>
-      <c r="D8" s="6" t="str">
+      <c r="D8" s="7" t="str">
         <f aca="false">'Spots Database'!C4</f>
         <v>Maine – North</v>
       </c>
-      <c r="E8" s="6" t="str">
+      <c r="E8" s="7" t="str">
         <f aca="false">'Spots Database'!E4</f>
         <v>Scarborough</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="7" t="str">
         <f aca="false">'Spots Database'!L4</f>
         <v>NE / E</v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="7" t="str">
         <f aca="false">'Spots Database'!M4</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H8" s="6" t="str">
+      <c r="H8" s="7" t="str">
         <f aca="false">'Spots Database'!O4</f>
         <v>Beach Break</v>
       </c>
-      <c r="I8" s="6" t="str">
+      <c r="I8" s="7" t="str">
         <f aca="false">'Spots Database'!P4</f>
         <v>Beginner–Int</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="str">
+      <c r="A9" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F5="Y"),AND($C$4="NE",'Spots Database'!G5="Y"),AND($C$4="E",'Spots Database'!H5="Y"),AND($C$4="SE",'Spots Database'!I5="Y"),AND($C$4="S",'Spots Database'!J5="Y"),AND($C$4="SW",'Spots Database'!K5="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B9" s="22" t="str">
+      <c r="B9" s="23" t="str">
         <f aca="false">'Spots Database'!S5</f>
         <v>★★★☆☆</v>
       </c>
-      <c r="C9" s="12" t="str">
+      <c r="C9" s="13" t="str">
         <f aca="false">'Spots Database'!B5</f>
         <v>Old Orchard Beach</v>
       </c>
-      <c r="D9" s="12" t="str">
+      <c r="D9" s="13" t="str">
         <f aca="false">'Spots Database'!C5</f>
         <v>Maine – North</v>
       </c>
-      <c r="E9" s="12" t="str">
+      <c r="E9" s="13" t="str">
         <f aca="false">'Spots Database'!E5</f>
         <v>Old Orchard Beach</v>
       </c>
-      <c r="F9" s="12" t="str">
+      <c r="F9" s="13" t="str">
         <f aca="false">'Spots Database'!L5</f>
         <v>NE / E / SE</v>
       </c>
-      <c r="G9" s="12" t="str">
+      <c r="G9" s="13" t="str">
         <f aca="false">'Spots Database'!M5</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H9" s="12" t="str">
+      <c r="H9" s="13" t="str">
         <f aca="false">'Spots Database'!O5</f>
         <v>Beach Break</v>
       </c>
-      <c r="I9" s="12" t="str">
+      <c r="I9" s="13" t="str">
         <f aca="false">'Spots Database'!P5</f>
         <v>Beginner</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="str">
+      <c r="A10" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F6="Y"),AND($C$4="NE",'Spots Database'!G6="Y"),AND($C$4="E",'Spots Database'!H6="Y"),AND($C$4="SE",'Spots Database'!I6="Y"),AND($C$4="S",'Spots Database'!J6="Y"),AND($C$4="SW",'Spots Database'!K6="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B10" s="22" t="str">
+      <c r="B10" s="23" t="str">
         <f aca="false">'Spots Database'!S6</f>
         <v>★★★☆☆</v>
       </c>
-      <c r="C10" s="6" t="str">
+      <c r="C10" s="7" t="str">
         <f aca="false">'Spots Database'!B6</f>
         <v>Scarborough Beach</v>
       </c>
-      <c r="D10" s="6" t="str">
+      <c r="D10" s="7" t="str">
         <f aca="false">'Spots Database'!C6</f>
         <v>Maine – North</v>
       </c>
-      <c r="E10" s="6" t="str">
+      <c r="E10" s="7" t="str">
         <f aca="false">'Spots Database'!E6</f>
         <v>Scarborough</v>
       </c>
-      <c r="F10" s="6" t="str">
+      <c r="F10" s="7" t="str">
         <f aca="false">'Spots Database'!L6</f>
         <v>NE / E</v>
       </c>
-      <c r="G10" s="6" t="str">
+      <c r="G10" s="7" t="str">
         <f aca="false">'Spots Database'!M6</f>
         <v>Mid</v>
       </c>
-      <c r="H10" s="6" t="str">
+      <c r="H10" s="7" t="str">
         <f aca="false">'Spots Database'!O6</f>
         <v>Beach Break</v>
       </c>
-      <c r="I10" s="6" t="str">
+      <c r="I10" s="7" t="str">
         <f aca="false">'Spots Database'!P6</f>
         <v>Intermediate</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="str">
+      <c r="A11" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F7="Y"),AND($C$4="NE",'Spots Database'!G7="Y"),AND($C$4="E",'Spots Database'!H7="Y"),AND($C$4="SE",'Spots Database'!I7="Y"),AND($C$4="S",'Spots Database'!J7="Y"),AND($C$4="SW",'Spots Database'!K7="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B11" s="22" t="str">
+      <c r="B11" s="23" t="str">
         <f aca="false">'Spots Database'!S7</f>
         <v>★★★☆☆</v>
       </c>
-      <c r="C11" s="12" t="str">
+      <c r="C11" s="13" t="str">
         <f aca="false">'Spots Database'!B7</f>
         <v>Fortunes Rocks Beach</v>
       </c>
-      <c r="D11" s="12" t="str">
+      <c r="D11" s="13" t="str">
         <f aca="false">'Spots Database'!C7</f>
         <v>Maine – North</v>
       </c>
-      <c r="E11" s="12" t="str">
+      <c r="E11" s="13" t="str">
         <f aca="false">'Spots Database'!E7</f>
         <v>Biddeford</v>
       </c>
-      <c r="F11" s="12" t="str">
+      <c r="F11" s="13" t="str">
         <f aca="false">'Spots Database'!L7</f>
         <v>NE / E</v>
       </c>
-      <c r="G11" s="12" t="str">
+      <c r="G11" s="13" t="str">
         <f aca="false">'Spots Database'!M7</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H11" s="12" t="str">
+      <c r="H11" s="13" t="str">
         <f aca="false">'Spots Database'!O7</f>
         <v>Beach Break</v>
       </c>
-      <c r="I11" s="12" t="str">
+      <c r="I11" s="13" t="str">
         <f aca="false">'Spots Database'!P7</f>
         <v>Beginner–Int</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="str">
+      <c r="A12" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F8="Y"),AND($C$4="NE",'Spots Database'!G8="Y"),AND($C$4="E",'Spots Database'!H8="Y"),AND($C$4="SE",'Spots Database'!I8="Y"),AND($C$4="S",'Spots Database'!J8="Y"),AND($C$4="SW",'Spots Database'!K8="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B12" s="22" t="str">
+      <c r="B12" s="23" t="str">
         <f aca="false">'Spots Database'!S8</f>
         <v>★★★☆☆</v>
       </c>
-      <c r="C12" s="6" t="str">
+      <c r="C12" s="7" t="str">
         <f aca="false">'Spots Database'!B8</f>
         <v>Kennebunk Beach</v>
       </c>
-      <c r="D12" s="6" t="str">
+      <c r="D12" s="7" t="str">
         <f aca="false">'Spots Database'!C8</f>
         <v>Maine – North</v>
       </c>
-      <c r="E12" s="6" t="str">
+      <c r="E12" s="7" t="str">
         <f aca="false">'Spots Database'!E8</f>
         <v>Kennebunk</v>
       </c>
-      <c r="F12" s="6" t="str">
+      <c r="F12" s="7" t="str">
         <f aca="false">'Spots Database'!L8</f>
         <v>NE / E</v>
       </c>
-      <c r="G12" s="6" t="str">
+      <c r="G12" s="7" t="str">
         <f aca="false">'Spots Database'!M8</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H12" s="6" t="str">
+      <c r="H12" s="7" t="str">
         <f aca="false">'Spots Database'!O8</f>
         <v>Beach Break</v>
       </c>
-      <c r="I12" s="6" t="str">
+      <c r="I12" s="7" t="str">
         <f aca="false">'Spots Database'!P8</f>
         <v>Intermediate</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="str">
+      <c r="A13" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F9="Y"),AND($C$4="NE",'Spots Database'!G9="Y"),AND($C$4="E",'Spots Database'!H9="Y"),AND($C$4="SE",'Spots Database'!I9="Y"),AND($C$4="S",'Spots Database'!J9="Y"),AND($C$4="SW",'Spots Database'!K9="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B13" s="22" t="str">
+      <c r="B13" s="23" t="str">
         <f aca="false">'Spots Database'!S9</f>
         <v>★★★☆☆</v>
       </c>
-      <c r="C13" s="12" t="str">
+      <c r="C13" s="13" t="str">
         <f aca="false">'Spots Database'!B9</f>
         <v>Kennebunkport</v>
       </c>
-      <c r="D13" s="12" t="str">
+      <c r="D13" s="13" t="str">
         <f aca="false">'Spots Database'!C9</f>
         <v>Maine – North</v>
       </c>
-      <c r="E13" s="12" t="str">
+      <c r="E13" s="13" t="str">
         <f aca="false">'Spots Database'!E9</f>
         <v>Kennebunkport</v>
       </c>
-      <c r="F13" s="12" t="str">
+      <c r="F13" s="13" t="str">
         <f aca="false">'Spots Database'!L9</f>
         <v>NE / E</v>
       </c>
-      <c r="G13" s="12" t="str">
+      <c r="G13" s="13" t="str">
         <f aca="false">'Spots Database'!M9</f>
         <v>Low</v>
       </c>
-      <c r="H13" s="12" t="str">
+      <c r="H13" s="13" t="str">
         <f aca="false">'Spots Database'!O9</f>
         <v>Beach Break</v>
       </c>
-      <c r="I13" s="12" t="str">
+      <c r="I13" s="13" t="str">
         <f aca="false">'Spots Database'!P9</f>
         <v>Intermediate</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="str">
+      <c r="A14" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F10="Y"),AND($C$4="NE",'Spots Database'!G10="Y"),AND($C$4="E",'Spots Database'!H10="Y"),AND($C$4="SE",'Spots Database'!I10="Y"),AND($C$4="S",'Spots Database'!J10="Y"),AND($C$4="SW",'Spots Database'!K10="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B14" s="22" t="str">
+      <c r="B14" s="23" t="str">
         <f aca="false">'Spots Database'!S10</f>
         <v>★★★★☆</v>
       </c>
-      <c r="C14" s="6" t="str">
+      <c r="C14" s="7" t="str">
         <f aca="false">'Spots Database'!B10</f>
         <v>Lox Point</v>
       </c>
-      <c r="D14" s="6" t="str">
+      <c r="D14" s="7" t="str">
         <f aca="false">'Spots Database'!C10</f>
         <v>Maine – North</v>
       </c>
-      <c r="E14" s="6" t="str">
+      <c r="E14" s="7" t="str">
         <f aca="false">'Spots Database'!E10</f>
         <v>Kennebunk</v>
       </c>
-      <c r="F14" s="6" t="str">
+      <c r="F14" s="7" t="str">
         <f aca="false">'Spots Database'!L10</f>
         <v>NE / E</v>
       </c>
-      <c r="G14" s="6" t="str">
+      <c r="G14" s="7" t="str">
         <f aca="false">'Spots Database'!M10</f>
         <v>Low</v>
       </c>
-      <c r="H14" s="6" t="str">
+      <c r="H14" s="7" t="str">
         <f aca="false">'Spots Database'!O10</f>
         <v>Point Break</v>
       </c>
-      <c r="I14" s="6" t="str">
+      <c r="I14" s="7" t="str">
         <f aca="false">'Spots Database'!P10</f>
         <v>Advanced</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="str">
+      <c r="A15" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F11="Y"),AND($C$4="NE",'Spots Database'!G11="Y"),AND($C$4="E",'Spots Database'!H11="Y"),AND($C$4="SE",'Spots Database'!I11="Y"),AND($C$4="S",'Spots Database'!J11="Y"),AND($C$4="SW",'Spots Database'!K11="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B15" s="22" t="str">
+      <c r="B15" s="23" t="str">
         <f aca="false">'Spots Database'!S11</f>
         <v>★★★★☆</v>
       </c>
-      <c r="C15" s="12" t="str">
+      <c r="C15" s="13" t="str">
         <f aca="false">'Spots Database'!B11</f>
         <v>Wells Jetties</v>
       </c>
-      <c r="D15" s="12" t="str">
+      <c r="D15" s="13" t="str">
         <f aca="false">'Spots Database'!C11</f>
         <v>Maine – South</v>
       </c>
-      <c r="E15" s="12" t="str">
+      <c r="E15" s="13" t="str">
         <f aca="false">'Spots Database'!E11</f>
         <v>Wells</v>
       </c>
-      <c r="F15" s="12" t="str">
+      <c r="F15" s="13" t="str">
         <f aca="false">'Spots Database'!L11</f>
         <v>NE / E</v>
       </c>
-      <c r="G15" s="12" t="str">
+      <c r="G15" s="13" t="str">
         <f aca="false">'Spots Database'!M11</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H15" s="12" t="str">
+      <c r="H15" s="13" t="str">
         <f aca="false">'Spots Database'!O11</f>
         <v>Jetty Break</v>
       </c>
-      <c r="I15" s="12" t="str">
+      <c r="I15" s="13" t="str">
         <f aca="false">'Spots Database'!P11</f>
         <v>Intermediate</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="str">
+      <c r="A16" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F12="Y"),AND($C$4="NE",'Spots Database'!G12="Y"),AND($C$4="E",'Spots Database'!H12="Y"),AND($C$4="SE",'Spots Database'!I12="Y"),AND($C$4="S",'Spots Database'!J12="Y"),AND($C$4="SW",'Spots Database'!K12="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B16" s="22" t="str">
+      <c r="B16" s="23" t="str">
         <f aca="false">'Spots Database'!S12</f>
         <v>★★☆☆☆</v>
       </c>
-      <c r="C16" s="6" t="str">
+      <c r="C16" s="7" t="str">
         <f aca="false">'Spots Database'!B12</f>
         <v>Wells Beach</v>
       </c>
-      <c r="D16" s="6" t="str">
+      <c r="D16" s="7" t="str">
         <f aca="false">'Spots Database'!C12</f>
         <v>Maine – South</v>
       </c>
-      <c r="E16" s="6" t="str">
+      <c r="E16" s="7" t="str">
         <f aca="false">'Spots Database'!E12</f>
         <v>Wells</v>
       </c>
-      <c r="F16" s="6" t="str">
+      <c r="F16" s="7" t="str">
         <f aca="false">'Spots Database'!L12</f>
         <v>NE / E</v>
       </c>
-      <c r="G16" s="6" t="str">
+      <c r="G16" s="7" t="str">
         <f aca="false">'Spots Database'!M12</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H16" s="6" t="str">
+      <c r="H16" s="7" t="str">
         <f aca="false">'Spots Database'!O12</f>
         <v>Beach Break</v>
       </c>
-      <c r="I16" s="6" t="str">
+      <c r="I16" s="7" t="str">
         <f aca="false">'Spots Database'!P12</f>
         <v>Beginner</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="str">
+      <c r="A17" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F13="Y"),AND($C$4="NE",'Spots Database'!G13="Y"),AND($C$4="E",'Spots Database'!H13="Y"),AND($C$4="SE",'Spots Database'!I13="Y"),AND($C$4="S",'Spots Database'!J13="Y"),AND($C$4="SW",'Spots Database'!K13="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B17" s="22" t="str">
+      <c r="B17" s="23" t="str">
         <f aca="false">'Spots Database'!S13</f>
         <v>★★☆☆☆</v>
       </c>
-      <c r="C17" s="12" t="str">
+      <c r="C17" s="13" t="str">
         <f aca="false">'Spots Database'!B13</f>
         <v>Moody Beach</v>
       </c>
-      <c r="D17" s="12" t="str">
+      <c r="D17" s="13" t="str">
         <f aca="false">'Spots Database'!C13</f>
         <v>Maine – South</v>
       </c>
-      <c r="E17" s="12" t="str">
+      <c r="E17" s="13" t="str">
         <f aca="false">'Spots Database'!E13</f>
         <v>Wells</v>
       </c>
-      <c r="F17" s="12" t="str">
+      <c r="F17" s="13" t="str">
         <f aca="false">'Spots Database'!L13</f>
         <v>NE / E</v>
       </c>
-      <c r="G17" s="12" t="str">
+      <c r="G17" s="13" t="str">
         <f aca="false">'Spots Database'!M13</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H17" s="12" t="str">
+      <c r="H17" s="13" t="str">
         <f aca="false">'Spots Database'!O13</f>
         <v>Beach Break</v>
       </c>
-      <c r="I17" s="12" t="str">
+      <c r="I17" s="13" t="str">
         <f aca="false">'Spots Database'!P13</f>
         <v>Beginner</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="str">
+      <c r="A18" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F14="Y"),AND($C$4="NE",'Spots Database'!G14="Y"),AND($C$4="E",'Spots Database'!H14="Y"),AND($C$4="SE",'Spots Database'!I14="Y"),AND($C$4="S",'Spots Database'!J14="Y"),AND($C$4="SW",'Spots Database'!K14="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B18" s="22" t="str">
+      <c r="B18" s="23" t="str">
         <f aca="false">'Spots Database'!S14</f>
         <v>★★★☆☆</v>
       </c>
-      <c r="C18" s="6" t="str">
+      <c r="C18" s="7" t="str">
         <f aca="false">'Spots Database'!B14</f>
         <v>Ogunquit Beach</v>
       </c>
-      <c r="D18" s="6" t="str">
+      <c r="D18" s="7" t="str">
         <f aca="false">'Spots Database'!C14</f>
         <v>Maine – South</v>
       </c>
-      <c r="E18" s="6" t="str">
+      <c r="E18" s="7" t="str">
         <f aca="false">'Spots Database'!E14</f>
         <v>Ogunquit</v>
       </c>
-      <c r="F18" s="6" t="str">
+      <c r="F18" s="7" t="str">
         <f aca="false">'Spots Database'!L14</f>
         <v>NE / E / SE</v>
       </c>
-      <c r="G18" s="6" t="str">
+      <c r="G18" s="7" t="str">
         <f aca="false">'Spots Database'!M14</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H18" s="6" t="str">
+      <c r="H18" s="7" t="str">
         <f aca="false">'Spots Database'!O14</f>
         <v>Beach Break</v>
       </c>
-      <c r="I18" s="6" t="str">
+      <c r="I18" s="7" t="str">
         <f aca="false">'Spots Database'!P14</f>
         <v>Beginner–Int</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="str">
+      <c r="A19" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F15="Y"),AND($C$4="NE",'Spots Database'!G15="Y"),AND($C$4="E",'Spots Database'!H15="Y"),AND($C$4="SE",'Spots Database'!I15="Y"),AND($C$4="S",'Spots Database'!J15="Y"),AND($C$4="SW",'Spots Database'!K15="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B19" s="22" t="str">
+      <c r="B19" s="23" t="str">
         <f aca="false">'Spots Database'!S15</f>
         <v>★★★★☆</v>
       </c>
-      <c r="C19" s="12" t="str">
+      <c r="C19" s="13" t="str">
         <f aca="false">'Spots Database'!B15</f>
         <v>Ogunquit Rivermouth</v>
       </c>
-      <c r="D19" s="12" t="str">
+      <c r="D19" s="13" t="str">
         <f aca="false">'Spots Database'!C15</f>
         <v>Maine – South</v>
       </c>
-      <c r="E19" s="12" t="str">
+      <c r="E19" s="13" t="str">
         <f aca="false">'Spots Database'!E15</f>
         <v>Ogunquit</v>
       </c>
-      <c r="F19" s="12" t="str">
+      <c r="F19" s="13" t="str">
         <f aca="false">'Spots Database'!L15</f>
         <v>NE / E / SE</v>
       </c>
-      <c r="G19" s="12" t="str">
+      <c r="G19" s="13" t="str">
         <f aca="false">'Spots Database'!M15</f>
         <v>Low</v>
       </c>
-      <c r="H19" s="12" t="str">
+      <c r="H19" s="13" t="str">
         <f aca="false">'Spots Database'!O15</f>
         <v>River Mouth</v>
       </c>
-      <c r="I19" s="12" t="str">
+      <c r="I19" s="13" t="str">
         <f aca="false">'Spots Database'!P15</f>
         <v>Intermediate–Adv</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="str">
+      <c r="A20" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F16="Y"),AND($C$4="NE",'Spots Database'!G16="Y"),AND($C$4="E",'Spots Database'!H16="Y"),AND($C$4="SE",'Spots Database'!I16="Y"),AND($C$4="S",'Spots Database'!J16="Y"),AND($C$4="SW",'Spots Database'!K16="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B20" s="22" t="str">
+      <c r="B20" s="23" t="str">
         <f aca="false">'Spots Database'!S16</f>
         <v>★★★★☆</v>
       </c>
-      <c r="C20" s="6" t="str">
+      <c r="C20" s="7" t="str">
         <f aca="false">'Spots Database'!B16</f>
         <v>Long Sands Beach</v>
       </c>
-      <c r="D20" s="6" t="str">
+      <c r="D20" s="7" t="str">
         <f aca="false">'Spots Database'!C16</f>
         <v>Maine – South</v>
       </c>
-      <c r="E20" s="6" t="str">
+      <c r="E20" s="7" t="str">
         <f aca="false">'Spots Database'!E16</f>
         <v>York</v>
       </c>
-      <c r="F20" s="6" t="str">
+      <c r="F20" s="7" t="str">
         <f aca="false">'Spots Database'!L16</f>
         <v>NE / E / SE</v>
       </c>
-      <c r="G20" s="6" t="str">
+      <c r="G20" s="7" t="str">
         <f aca="false">'Spots Database'!M16</f>
         <v>Low–Mid</v>
       </c>
-      <c r="H20" s="6" t="str">
+      <c r="H20" s="7" t="str">
         <f aca="false">'Spots Database'!O16</f>
         <v>Beach Break</v>
       </c>
-      <c r="I20" s="6" t="str">
+      <c r="I20" s="7" t="str">
         <f aca="false">'Spots Database'!P16</f>
         <v>Beginner–Int</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="str">
+      <c r="A21" s="22" t="str">
         <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F17="Y"),AND($C$4="NE",'Spots Database'!G17="Y"),AND($C$4="E",'Spots Database'!H17="Y"),AND($C$4="SE",'Spots Database'!I17="Y"),AND($C$4="S",'Spots Database'!J17="Y"),AND($C$4="SW",'Spots Database'!K17="Y")),"✅","—")</f>
         <v>✅</v>
       </c>
-      <c r="B21" s="22" t="str">
+      <c r="B21" s="23" t="str">
         <f aca="false">'Spots Database'!S17</f>
         <v>★★★☆☆</v>
       </c>
-      <c r="C21" s="12" t="str">
+      <c r="C21" s="13" t="str">
         <f aca="false">'Spots Database'!B17</f>
         <v>Short Sands Beach</v>
       </c>
-      <c r="D21" s="12" t="str">
+      <c r="D21" s="13" t="str">
         <f aca="false">'Spots Database'!C17</f>
         <v>Maine – South</v>
       </c>
-      <c r="E21" s="12" t="str">
+      <c r="E21" s="13" t="str">
         <f aca="false">'Spots Database'!E17</f>
         <v>York</v>
       </c>
-      <c r="F21" s="12" t="str">
+      <c r="F21" s="13" t="str">
         <f aca="false">'Spots Database'!L17</f>
         <v>NE / E / SE</v>
       </c>
-      <c r="G21" s="12" t="str">
+      <c r="G21" s="13" t="str">
         <f aca="false">'Spots Database'!M17</f>
         <v>All Tides</v>
       </c>
-      <c r="H21" s="12" t="str">
+      <c r="H21" s="13" t="str">
         <f aca="false">'Spots Database'!O17</f>
         <v>Beach Break</v>
       </c>
-      <c r="I21" s="12" t="str">
+      <c r="I21" s="13" t="str">
         <f aca="false">'Spots Database'!P17</f>
         <v>Beginner</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="str">
+        <f aca="false">IF(OR(AND($C$4="N",'Spots Database'!F18="Y"),AND($C$4="NE",'Spots Database'!G18="Y"),AND($C$4="E",'Spots Database'!H18="Y"),AND($C$4="SE",'Spots Database'!I18="Y"),AND($C$4="S",'Spots Database'!J18="Y"),AND($C$4="SW",'Spots Database'!K18="Y")),"✅","—")</f>
+        <v>✅</v>
+      </c>
+      <c r="B22" s="23" t="str">
+        <f aca="false">'Spots Database'!S18</f>
+        <v>★★★★☆</v>
+      </c>
+      <c r="C22" s="25" t="str">
+        <f aca="false">'Spots Database'!B18</f>
+        <v>Pine Point</v>
+      </c>
+      <c r="D22" s="25" t="str">
+        <f aca="false">'Spots Database'!C18</f>
+        <v>Maine – North</v>
+      </c>
+      <c r="E22" s="25" t="str">
+        <f aca="false">'Spots Database'!E18</f>
+        <v>Scarborough</v>
+      </c>
+      <c r="F22" s="25" t="str">
+        <f aca="false">'Spots Database'!L18</f>
+        <v>NE / E</v>
+      </c>
+      <c r="G22" s="25" t="str">
+        <f aca="false">'Spots Database'!M18</f>
+        <v>Low</v>
+      </c>
+      <c r="H22" s="25" t="str">
+        <f aca="false">'Spots Database'!O18</f>
+        <v>River Mouth</v>
+      </c>
+      <c r="I22" s="25" t="str">
+        <f aca="false">'Spots Database'!P18</f>
+        <v>Intermediate</v>
+      </c>
+    </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="23"/>
+      <c r="A23" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2879,115 +3032,123 @@
     <mergeCell ref="A23:I23"/>
   </mergeCells>
   <conditionalFormatting sqref="A8:I8">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A8="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A8="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9:I9">
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A9="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A9="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10:I10">
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A10="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A10="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A11:I11">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A11="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A11="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A12:I12">
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A12="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A12="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13:I13">
-    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A13="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A13="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:I14">
-    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A14="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A14="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A15:I15">
-    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A15="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A15="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:I16">
-    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A16="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A16="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A17:I17">
-    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A17="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A17="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18:I18">
-    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A18="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A18="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A19:I19">
-    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A19="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A19="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20:I20">
-    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A20="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A20="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:I21">
-    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$A21="✅"</formula>
     </cfRule>
-    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$A21="—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A22:I22">
+    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+      <formula>$A22="✅"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+      <formula>$A22="—"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -3015,195 +3176,195 @@
   <dimension ref="A1:B26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="2"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24" t="s">
-        <v>94</v>
-      </c>
-      <c r="B1" s="24"/>
+      <c r="A1" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="27"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" s="25"/>
+      <c r="A2" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" s="28"/>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>97</v>
+      <c r="A3" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>99</v>
+      <c r="A4" s="31" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>100</v>
-      </c>
-      <c r="B5" s="27" t="s">
-        <v>101</v>
+      <c r="A5" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>103</v>
+      <c r="A6" s="31" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="30"/>
-      <c r="B7" s="30"/>
+      <c r="A7" s="33"/>
+      <c r="B7" s="33"/>
     </row>
     <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" s="25"/>
+      <c r="A8" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8" s="28"/>
     </row>
     <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" s="27" t="s">
-        <v>106</v>
+      <c r="A9" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
-        <v>107</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>108</v>
+      <c r="A10" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
-        <v>109</v>
-      </c>
-      <c r="B11" s="27" t="s">
-        <v>110</v>
+      <c r="A11" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
-        <v>111</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>112</v>
+      <c r="A12" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="26" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="27" t="s">
-        <v>114</v>
+      <c r="A13" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
-        <v>115</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>116</v>
+      <c r="A14" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" s="32" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="30"/>
-      <c r="B15" s="30"/>
+      <c r="A15" s="33"/>
+      <c r="B15" s="33"/>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="B16" s="25"/>
+      <c r="A16" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="28"/>
     </row>
     <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="27" t="s">
-        <v>118</v>
+      <c r="B17" s="30" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="29" t="s">
-        <v>119</v>
+      <c r="B18" s="32" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="27" t="s">
-        <v>120</v>
+      <c r="B19" s="30" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="29" t="s">
-        <v>121</v>
+      <c r="B20" s="32" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="26" t="s">
+      <c r="A21" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="27" t="s">
-        <v>122</v>
+      <c r="B21" s="30" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="29" t="s">
-        <v>123</v>
+      <c r="B22" s="32" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="30"/>
-      <c r="B23" s="30"/>
+      <c r="A23" s="33"/>
+      <c r="B23" s="33"/>
     </row>
     <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="B24" s="25"/>
+      <c r="A24" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="28"/>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="s">
-        <v>125</v>
-      </c>
-      <c r="B25" s="27" t="s">
-        <v>126</v>
+      <c r="A25" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="30" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28" t="s">
-        <v>127</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>128</v>
+      <c r="A26" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="B26" s="32" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>